<commit_message>
added: demographic report excel
</commit_message>
<xml_diff>
--- a/storage/app/template/List-of-all-Applicant.xlsx
+++ b/storage/app/template/List-of-all-Applicant.xlsx
@@ -8,12 +8,13 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\cenro\Deniel\RSP-Docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D46DFE19-8300-45B1-ACB8-AE36B098BCCE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3BA12352-1EF5-46D1-82CD-2261AF1C82F6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="23520" xr2:uid="{8113A99E-9156-40D8-A2D8-36A56E68640F}"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="List" sheetId="1" r:id="rId1"/>
+    <sheet name="Summary" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -34,7 +35,10 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="13" uniqueCount="13">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="34" uniqueCount="28">
+  <si>
+    <t>GENDER</t>
+  </si>
   <si>
     <t>NO.</t>
   </si>
@@ -42,6 +46,9 @@
     <t>NAME</t>
   </si>
   <si>
+    <t>POSITION APPLIED</t>
+  </si>
+  <si>
     <t>POSITION LEVEL</t>
   </si>
   <si>
@@ -51,9 +58,6 @@
     <t>SG</t>
   </si>
   <si>
-    <t>GENDER</t>
-  </si>
-  <si>
     <t>CIVIL STATUS</t>
   </si>
   <si>
@@ -66,20 +70,62 @@
     <t>PWD</t>
   </si>
   <si>
-    <t xml:space="preserve">LIST OF ALL APPLICANT </t>
-  </si>
-  <si>
-    <t>POSITION APPLIED</t>
-  </si>
-  <si>
-    <t>PUBLICATION DATE:</t>
+    <t xml:space="preserve">PUBLICATION DATE: </t>
+  </si>
+  <si>
+    <t>LIST OF ALL APPLICANTIONS</t>
+  </si>
+  <si>
+    <t>Variable</t>
+  </si>
+  <si>
+    <t>Gender</t>
+  </si>
+  <si>
+    <t>Male</t>
+  </si>
+  <si>
+    <t>Female</t>
+  </si>
+  <si>
+    <t>Civil Status</t>
+  </si>
+  <si>
+    <t>Single</t>
+  </si>
+  <si>
+    <t>Separated</t>
+  </si>
+  <si>
+    <t>Married</t>
+  </si>
+  <si>
+    <t>Solo Parent</t>
+  </si>
+  <si>
+    <t>IP</t>
+  </si>
+  <si>
+    <t>Category</t>
+  </si>
+  <si>
+    <t>Yes</t>
+  </si>
+  <si>
+    <t>No</t>
+  </si>
+  <si>
+    <t>Count</t>
+  </si>
+  <si>
+    <t>DEMOGRAPHIC</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="5" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -100,21 +146,55 @@
       <name val="Aptos"/>
       <family val="2"/>
     </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FF000000"/>
+      <name val="Aptos"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="10"/>
+      <color rgb="FF000000"/>
+      <name val="Aptos"/>
+      <family val="2"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="2"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="2">
+  <borders count="3">
     <border>
       <left/>
       <right/>
       <top/>
       <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF000000"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF000000"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF000000"/>
+      </bottom>
       <diagonal/>
     </border>
     <border>
@@ -136,31 +216,59 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="19">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -476,87 +584,139 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A02B2E2A-17B3-4664-9767-1B738A9DDE6E}">
-  <dimension ref="A2:K6"/>
+  <dimension ref="A1:K8"/>
   <sheetFormatPr defaultRowHeight="13.5" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="9.140625" style="7"/>
-    <col min="2" max="2" width="32.7109375" style="8" customWidth="1"/>
-    <col min="3" max="3" width="42.28515625" style="8" customWidth="1"/>
-    <col min="4" max="4" width="13.28515625" style="7" customWidth="1"/>
-    <col min="5" max="5" width="22.28515625" style="7" customWidth="1"/>
-    <col min="6" max="6" width="13" style="6" customWidth="1"/>
-    <col min="7" max="7" width="15" style="7" customWidth="1"/>
-    <col min="8" max="8" width="14.5703125" style="7" customWidth="1"/>
-    <col min="9" max="9" width="39.28515625" style="8" customWidth="1"/>
-    <col min="10" max="10" width="19.140625" style="7" customWidth="1"/>
-    <col min="11" max="11" width="13.42578125" style="7" customWidth="1"/>
-    <col min="12" max="16384" width="9.140625" style="3"/>
+    <col min="1" max="1" width="9.140625" style="1"/>
+    <col min="2" max="2" width="32.7109375" style="2" customWidth="1"/>
+    <col min="3" max="3" width="42.28515625" style="2" customWidth="1"/>
+    <col min="4" max="4" width="13.28515625" style="1" customWidth="1"/>
+    <col min="5" max="5" width="22.28515625" style="1" customWidth="1"/>
+    <col min="6" max="6" width="13" style="1" customWidth="1"/>
+    <col min="7" max="7" width="15" style="1" customWidth="1"/>
+    <col min="8" max="8" width="14.5703125" style="1" customWidth="1"/>
+    <col min="9" max="9" width="39.28515625" style="2" customWidth="1"/>
+    <col min="10" max="10" width="19.140625" style="1" customWidth="1"/>
+    <col min="11" max="11" width="13.42578125" style="1" customWidth="1"/>
+    <col min="12" max="16384" width="9.140625" style="18"/>
   </cols>
   <sheetData>
-    <row r="2" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A2" s="2" t="s">
+    <row r="1" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A1" s="3"/>
+      <c r="B1" s="4"/>
+      <c r="C1" s="4"/>
+      <c r="D1" s="3"/>
+      <c r="E1" s="3"/>
+      <c r="F1" s="3"/>
+      <c r="G1" s="3"/>
+      <c r="H1" s="3"/>
+      <c r="I1" s="4"/>
+      <c r="J1" s="3"/>
+      <c r="K1" s="3"/>
+    </row>
+    <row r="2" spans="1:11" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A2" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="B2" s="5"/>
+      <c r="C2" s="5"/>
+      <c r="D2" s="5"/>
+      <c r="E2" s="5"/>
+      <c r="F2" s="5"/>
+      <c r="G2" s="5"/>
+      <c r="H2" s="5"/>
+      <c r="I2" s="5"/>
+      <c r="J2" s="5"/>
+      <c r="K2" s="5"/>
+    </row>
+    <row r="3" spans="1:11" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A3" s="5" t="s">
+        <v>11</v>
+      </c>
+      <c r="B3" s="11"/>
+      <c r="C3" s="11"/>
+      <c r="D3" s="11"/>
+      <c r="E3" s="11"/>
+      <c r="F3" s="11"/>
+      <c r="G3" s="11"/>
+      <c r="H3" s="11"/>
+      <c r="I3" s="11"/>
+      <c r="J3" s="11"/>
+      <c r="K3" s="11"/>
+    </row>
+    <row r="4" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A4" s="3"/>
+      <c r="B4" s="4"/>
+      <c r="C4" s="4"/>
+      <c r="D4" s="3"/>
+      <c r="E4" s="3"/>
+      <c r="F4" s="3"/>
+      <c r="G4" s="3"/>
+      <c r="H4" s="3"/>
+      <c r="I4" s="4"/>
+      <c r="J4" s="3"/>
+      <c r="K4" s="3"/>
+    </row>
+    <row r="5" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A5" s="3"/>
+      <c r="B5" s="4"/>
+      <c r="C5" s="4"/>
+      <c r="D5" s="3"/>
+      <c r="E5" s="3"/>
+      <c r="F5" s="3"/>
+      <c r="G5" s="3"/>
+      <c r="H5" s="3"/>
+      <c r="I5" s="4"/>
+      <c r="J5" s="3"/>
+      <c r="K5" s="3"/>
+    </row>
+    <row r="6" spans="1:11" ht="40.5" x14ac:dyDescent="0.25">
+      <c r="A6" s="7" t="s">
+        <v>1</v>
+      </c>
+      <c r="B6" s="7" t="s">
+        <v>2</v>
+      </c>
+      <c r="C6" s="7" t="s">
+        <v>3</v>
+      </c>
+      <c r="D6" s="7" t="s">
+        <v>4</v>
+      </c>
+      <c r="E6" s="7" t="s">
+        <v>5</v>
+      </c>
+      <c r="F6" s="7" t="s">
+        <v>6</v>
+      </c>
+      <c r="G6" s="7" t="s">
+        <v>0</v>
+      </c>
+      <c r="H6" s="7" t="s">
+        <v>7</v>
+      </c>
+      <c r="I6" s="7" t="s">
+        <v>8</v>
+      </c>
+      <c r="J6" s="7" t="s">
+        <v>9</v>
+      </c>
+      <c r="K6" s="7" t="s">
         <v>10</v>
       </c>
-      <c r="B2" s="2"/>
-      <c r="C2" s="2"/>
-      <c r="D2" s="2"/>
-      <c r="E2" s="2"/>
-      <c r="F2" s="2"/>
-      <c r="G2" s="2"/>
-      <c r="H2" s="2"/>
-      <c r="I2" s="2"/>
-      <c r="J2" s="2"/>
-      <c r="K2" s="2"/>
-    </row>
-    <row r="3" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A3" s="4" t="s">
-        <v>12</v>
-      </c>
-      <c r="B3" s="5"/>
-      <c r="C3" s="5"/>
-      <c r="D3" s="5"/>
-      <c r="E3" s="5"/>
-      <c r="F3" s="5"/>
-      <c r="G3" s="5"/>
-      <c r="H3" s="5"/>
-      <c r="I3" s="5"/>
-      <c r="J3" s="5"/>
-      <c r="K3" s="5"/>
-    </row>
-    <row r="6" spans="1:11" ht="40.5" x14ac:dyDescent="0.25">
-      <c r="A6" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B6" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C6" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="D6" s="1" t="s">
-        <v>2</v>
-      </c>
-      <c r="E6" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="F6" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="G6" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="H6" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="I6" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="J6" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="K6" s="1" t="s">
-        <v>9</v>
-      </c>
+    </row>
+    <row r="8" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A8" s="8"/>
+      <c r="B8" s="8"/>
+      <c r="C8" s="8"/>
+      <c r="D8" s="8"/>
+      <c r="E8" s="8"/>
+      <c r="F8" s="8"/>
+      <c r="G8" s="8"/>
+      <c r="H8" s="8"/>
+      <c r="I8" s="8"/>
+      <c r="J8" s="8"/>
+      <c r="K8" s="8"/>
     </row>
   </sheetData>
   <mergeCells count="2">
@@ -565,4 +725,152 @@
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7136F0B3-94F4-496F-9310-450264673E9D}">
+  <dimension ref="B2:L16"/>
+  <sheetFormatPr defaultRowHeight="13.5" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="9.140625" style="13"/>
+    <col min="2" max="2" width="18.28515625" style="10" customWidth="1"/>
+    <col min="3" max="3" width="29.28515625" style="13" customWidth="1"/>
+    <col min="4" max="16384" width="9.140625" style="13"/>
+  </cols>
+  <sheetData>
+    <row r="2" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="B2" s="6" t="s">
+        <v>27</v>
+      </c>
+      <c r="C2" s="6"/>
+      <c r="D2" s="6"/>
+      <c r="E2" s="12"/>
+      <c r="F2" s="12"/>
+      <c r="G2" s="12"/>
+      <c r="H2" s="12"/>
+      <c r="I2" s="12"/>
+      <c r="J2" s="12"/>
+      <c r="K2" s="12"/>
+      <c r="L2" s="12"/>
+    </row>
+    <row r="3" spans="2:12" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B3" s="6" t="s">
+        <v>11</v>
+      </c>
+      <c r="C3" s="6"/>
+      <c r="D3" s="6"/>
+      <c r="E3" s="14"/>
+      <c r="F3" s="14"/>
+      <c r="G3" s="14"/>
+      <c r="H3" s="14"/>
+      <c r="I3" s="14"/>
+      <c r="J3" s="14"/>
+      <c r="K3" s="14"/>
+      <c r="L3" s="14"/>
+    </row>
+    <row r="5" spans="2:12" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B5" s="15" t="s">
+        <v>13</v>
+      </c>
+      <c r="C5" s="15" t="s">
+        <v>23</v>
+      </c>
+      <c r="D5" s="16" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="6" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="B6" s="17" t="s">
+        <v>14</v>
+      </c>
+      <c r="C6" s="17" t="s">
+        <v>15</v>
+      </c>
+      <c r="D6" s="9"/>
+    </row>
+    <row r="7" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="B7" s="17"/>
+      <c r="C7" s="17" t="s">
+        <v>16</v>
+      </c>
+      <c r="D7" s="9"/>
+    </row>
+    <row r="8" spans="2:12" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B8" s="17" t="s">
+        <v>17</v>
+      </c>
+      <c r="C8" s="17" t="s">
+        <v>18</v>
+      </c>
+      <c r="D8" s="9"/>
+    </row>
+    <row r="9" spans="2:12" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B9" s="17"/>
+      <c r="C9" s="17" t="s">
+        <v>20</v>
+      </c>
+      <c r="D9" s="9"/>
+    </row>
+    <row r="10" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="B10" s="17"/>
+      <c r="C10" s="17" t="s">
+        <v>19</v>
+      </c>
+      <c r="D10" s="9"/>
+    </row>
+    <row r="11" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="B11" s="17" t="s">
+        <v>22</v>
+      </c>
+      <c r="C11" s="17" t="s">
+        <v>24</v>
+      </c>
+      <c r="D11" s="9"/>
+    </row>
+    <row r="12" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="B12" s="17"/>
+      <c r="C12" s="17" t="s">
+        <v>25</v>
+      </c>
+      <c r="D12" s="9"/>
+    </row>
+    <row r="13" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="B13" s="17" t="s">
+        <v>21</v>
+      </c>
+      <c r="C13" s="17" t="s">
+        <v>24</v>
+      </c>
+      <c r="D13" s="9"/>
+    </row>
+    <row r="14" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="B14" s="17"/>
+      <c r="C14" s="17" t="s">
+        <v>25</v>
+      </c>
+      <c r="D14" s="9"/>
+    </row>
+    <row r="15" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="B15" s="17" t="s">
+        <v>10</v>
+      </c>
+      <c r="C15" s="17" t="s">
+        <v>24</v>
+      </c>
+      <c r="D15" s="9"/>
+    </row>
+    <row r="16" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="B16" s="17"/>
+      <c r="C16" s="17" t="s">
+        <v>25</v>
+      </c>
+      <c r="D16" s="9"/>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="B2:D2"/>
+    <mergeCell ref="B3:D3"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>